<commit_message>
Beauty priority sheet: move Oura, Philips, Wilkinson Sword, Therabody to do-not-approach (current F1 sponsors)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TE8a9ptd2NGPUtY6iZfzkb
</commit_message>
<xml_diff>
--- a/reports/F1-Beauty-x-F1-Priority-2026-10.xlsx
+++ b/reports/F1-Beauty-x-F1-Priority-2026-10.xlsx
@@ -1157,17 +1157,17 @@
       <c r="K15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>A - approach first</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>~USD 11B valuation (2025), Team USA/Team Finland official wearable. Had a 2020 Red Bull Racing deal that appears lapsed: confirm before outreach. WHOOP owns Ferrari so the category is contested.</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>X - do not approach (F1 tie / no capacity)</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a current F1 sponsor in the August sponsor map. Already in F1: do not approach as a new prospect.</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
         <is>
           <t>Oura</t>
         </is>
@@ -3765,17 +3765,17 @@
       <c r="K67" s="4" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="5" t="inlineStr">
-        <is>
-          <t>B - approach with caveat</t>
-        </is>
-      </c>
-      <c r="B68" s="5" t="inlineStr">
-        <is>
-          <t>Edgewell-owned (listed ~USD 2B, no F1 tie); razors face Gillette/Audi head-on, which is a pitch angle.</t>
-        </is>
-      </c>
-      <c r="C68" s="5" t="inlineStr">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>X - do not approach (F1 tie / no capacity)</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a current F1 sponsor (Edgewell) in the August sponsor map. Already in F1.</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
         <is>
           <t>Wilkinson Sword</t>
         </is>
@@ -4459,17 +4459,17 @@
       <c r="K81" s="4" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="A82" s="5" t="inlineStr">
-        <is>
-          <t>B - approach with caveat</t>
-        </is>
-      </c>
-      <c r="B82" s="5" t="inlineStr">
-        <is>
-          <t>Was Red Bull Racing official recovery partner (2021), appears lapsed: confirm before outreach. Strong fit otherwise.</t>
-        </is>
-      </c>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="A82" s="7" t="inlineStr">
+        <is>
+          <t>X - do not approach (F1 tie / no capacity)</t>
+        </is>
+      </c>
+      <c r="B82" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a current F1 sponsor in the August sponsor map. Already in F1.</t>
+        </is>
+      </c>
+      <c r="C82" s="7" t="inlineStr">
         <is>
           <t>Therabody</t>
         </is>
@@ -5541,17 +5541,17 @@
       <c r="K103" s="4" t="inlineStr"/>
     </row>
     <row r="104">
-      <c r="A104" s="6" t="inlineStr">
-        <is>
-          <t>C - low priority</t>
-        </is>
-      </c>
-      <c r="B104" s="6" t="inlineStr">
-        <is>
-          <t>Listed (~EUR 20B), no F1 tie; grooming/beauty is a small division of a health-tech group.</t>
-        </is>
-      </c>
-      <c r="C104" s="6" t="inlineStr">
+      <c r="A104" s="7" t="inlineStr">
+        <is>
+          <t>X - do not approach (F1 tie / no capacity)</t>
+        </is>
+      </c>
+      <c r="B104" s="7" t="inlineStr">
+        <is>
+          <t>Listed as a current F1 sponsor in the August sponsor map. Already in F1.</t>
+        </is>
+      </c>
+      <c r="C104" s="7" t="inlineStr">
         <is>
           <t>Philips</t>
         </is>

</xml_diff>